<commit_message>
nick changes to figures
</commit_message>
<xml_diff>
--- a/fibre_analysis_output.xlsx
+++ b/fibre_analysis_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:Y10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -874,316 +874,395 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1812222222222222</v>
+        <v>0.1019477222222222</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01793246743209137</v>
+        <v>0.02806571590533813</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1458888888888889</v>
+        <v>0.05956988888888887</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2101111111111111</v>
+        <v>0.1609652222222222</v>
       </c>
       <c r="F6" t="n">
-        <v>321.9292714531197</v>
+        <v>262.2349577519491</v>
       </c>
       <c r="G6" t="n">
-        <v>46.12942604802129</v>
+        <v>95.83139734659412</v>
       </c>
       <c r="H6" t="n">
-        <v>230.0600840540321</v>
+        <v>142.7512275889141</v>
       </c>
       <c r="I6" t="n">
-        <v>414.0804550085159</v>
+        <v>429.7672182778938</v>
       </c>
       <c r="J6" t="n">
-        <v>14.32905614323387</v>
+        <v>36.54409700679268</v>
       </c>
       <c r="K6" t="n">
-        <v>9.895291654740795</v>
+        <v>27.5295173777021</v>
       </c>
       <c r="L6" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="M6" t="n">
-        <v>341.5299426664553</v>
+        <v>294.4214598098467</v>
       </c>
       <c r="N6" t="n">
-        <v>362.8538496905764</v>
+        <v>366.4463652708171</v>
       </c>
       <c r="O6" t="n">
-        <v>321.4591820845206</v>
+        <v>236.5530244310066</v>
       </c>
       <c r="P6" t="n">
-        <v>7.874640717792407</v>
+        <v>3.000674472344666</v>
       </c>
       <c r="Q6" t="n">
-        <v>11.03848404409053</v>
+        <v>4.831077348550521</v>
       </c>
       <c r="R6" t="n">
-        <v>5.617616167820732</v>
+        <v>1.863776263421335</v>
       </c>
       <c r="S6" t="n">
-        <v>234.2175761558871</v>
+        <v>109.4173790282314</v>
       </c>
       <c r="T6" t="n">
-        <v>1.360231578947368</v>
+        <v>1.02264</v>
       </c>
       <c r="U6" t="n">
-        <v>0.3568554345524118</v>
+        <v>0.3159439725295892</v>
       </c>
       <c r="V6" t="n">
-        <v>29.20044100328285</v>
+        <v>29.59462872760919</v>
       </c>
       <c r="W6" t="n">
-        <v>2.70308564432637</v>
+        <v>7.654014898946032</v>
       </c>
       <c r="X6" t="n">
-        <v>26.23490294414195</v>
+        <v>30.89493590409031</v>
       </c>
       <c r="Y6" t="n">
-        <v>9.25700281041124</v>
+        <v>25.86285156470137</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>X1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.229375</v>
+        <v>0.1812222222222222</v>
       </c>
       <c r="C7" t="n">
-        <v>0.02271454152795949</v>
+        <v>0.01793246743209137</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2026666666666667</v>
+        <v>0.1458888888888889</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2695555555555555</v>
+        <v>0.2101111111111111</v>
       </c>
       <c r="F7" t="n">
-        <v>231.6500536459821</v>
+        <v>321.9292714531197</v>
       </c>
       <c r="G7" t="n">
-        <v>54.91333296088788</v>
+        <v>46.12942604802129</v>
       </c>
       <c r="H7" t="n">
-        <v>148.42154728971</v>
+        <v>230.0600840540321</v>
       </c>
       <c r="I7" t="n">
-        <v>303.3232514860957</v>
+        <v>414.0804550085159</v>
       </c>
       <c r="J7" t="n">
-        <v>23.7052968892504</v>
+        <v>14.32905614323387</v>
       </c>
       <c r="K7" t="n">
-        <v>9.902797396385608</v>
+        <v>9.895291654740795</v>
       </c>
       <c r="L7" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="M7" t="n">
-        <v>253.5339625576554</v>
+        <v>341.5299426664553</v>
       </c>
       <c r="N7" t="n">
-        <v>300.1600884723132</v>
+        <v>362.8538496905764</v>
       </c>
       <c r="O7" t="n">
-        <v>214.1506237466203</v>
+        <v>321.4591820845206</v>
       </c>
       <c r="P7" t="n">
-        <v>4.370722856273517</v>
+        <v>7.874640717792407</v>
       </c>
       <c r="Q7" t="n">
-        <v>7.861448503708708</v>
+        <v>11.03848404409053</v>
       </c>
       <c r="R7" t="n">
-        <v>2.429987079014715</v>
+        <v>5.617616167820732</v>
       </c>
       <c r="S7" t="n">
-        <v>128.5003529794584</v>
+        <v>234.2175761558871</v>
       </c>
       <c r="T7" t="n">
-        <v>1.16765</v>
+        <v>1.360231578947368</v>
       </c>
       <c r="U7" t="n">
-        <v>0.3615817591796199</v>
+        <v>0.3568554345524118</v>
       </c>
       <c r="V7" t="n">
-        <v>25.41860227555073</v>
+        <v>29.20044100328285</v>
       </c>
       <c r="W7" t="n">
-        <v>2.439075284771629</v>
+        <v>2.70308564432637</v>
       </c>
       <c r="X7" t="n">
-        <v>30.96662177704105</v>
+        <v>26.23490294414195</v>
       </c>
       <c r="Y7" t="n">
-        <v>9.59563101987591</v>
+        <v>9.25700281041124</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3024912280701755</v>
+        <v>0.229375</v>
       </c>
       <c r="C8" t="n">
-        <v>0.02889915097384144</v>
+        <v>0.02271454152795949</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2511111111111111</v>
+        <v>0.2026666666666667</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3657777777777778</v>
+        <v>0.2695555555555555</v>
       </c>
       <c r="F8" t="n">
-        <v>233.3046299789876</v>
+        <v>231.6500536459821</v>
       </c>
       <c r="G8" t="n">
-        <v>37.15536440938772</v>
+        <v>54.91333296088788</v>
       </c>
       <c r="H8" t="n">
-        <v>172.5419493131833</v>
+        <v>148.42154728971</v>
       </c>
       <c r="I8" t="n">
-        <v>299.1806953288255</v>
+        <v>303.3232514860957</v>
       </c>
       <c r="J8" t="n">
-        <v>15.92568669243045</v>
+        <v>23.7052968892504</v>
       </c>
       <c r="K8" t="n">
-        <v>9.553715378198364</v>
+        <v>9.902797396385608</v>
       </c>
       <c r="L8" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="M8" t="n">
-        <v>248.8597278197844</v>
+        <v>253.5339625576554</v>
       </c>
       <c r="N8" t="n">
-        <v>266.1408330225629</v>
+        <v>300.1600884723132</v>
       </c>
       <c r="O8" t="n">
-        <v>232.7007224978768</v>
+        <v>214.1506237466203</v>
       </c>
       <c r="P8" t="n">
-        <v>7.079256509416166</v>
+        <v>4.370722856273517</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.01760915119143</v>
+        <v>7.861448503708708</v>
       </c>
       <c r="R8" t="n">
-        <v>5.002777805535633</v>
+        <v>2.429987079014715</v>
       </c>
       <c r="S8" t="n">
-        <v>163.583936740707</v>
+        <v>128.5003529794584</v>
       </c>
       <c r="T8" t="n">
-        <v>1.820252631578947</v>
+        <v>1.16765</v>
       </c>
       <c r="U8" t="n">
-        <v>0.441002679972231</v>
+        <v>0.3615817591796199</v>
       </c>
       <c r="V8" t="n">
-        <v>17.95502003555078</v>
+        <v>25.41860227555073</v>
       </c>
       <c r="W8" t="n">
-        <v>2.044232555680449</v>
+        <v>2.439075284771629</v>
       </c>
       <c r="X8" t="n">
-        <v>24.22755349018178</v>
+        <v>30.96662177704105</v>
       </c>
       <c r="Y8" t="n">
-        <v>11.38529810400037</v>
+        <v>9.59563101987591</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3024912280701755</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.02889915097384144</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2511111111111111</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3657777777777778</v>
+      </c>
+      <c r="F9" t="n">
+        <v>233.3046299789876</v>
+      </c>
+      <c r="G9" t="n">
+        <v>37.15536440938772</v>
+      </c>
+      <c r="H9" t="n">
+        <v>172.5419493131833</v>
+      </c>
+      <c r="I9" t="n">
+        <v>299.1806953288255</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15.92568669243045</v>
+      </c>
+      <c r="K9" t="n">
+        <v>9.553715378198364</v>
+      </c>
+      <c r="L9" t="n">
+        <v>19</v>
+      </c>
+      <c r="M9" t="n">
+        <v>248.8597278197844</v>
+      </c>
+      <c r="N9" t="n">
+        <v>266.1408330225629</v>
+      </c>
+      <c r="O9" t="n">
+        <v>232.7007224978768</v>
+      </c>
+      <c r="P9" t="n">
+        <v>7.079256509416166</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>10.01760915119143</v>
+      </c>
+      <c r="R9" t="n">
+        <v>5.002777805535633</v>
+      </c>
+      <c r="S9" t="n">
+        <v>163.583936740707</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.820252631578947</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.441002679972231</v>
+      </c>
+      <c r="V9" t="n">
+        <v>17.95502003555078</v>
+      </c>
+      <c r="W9" t="n">
+        <v>2.044232555680449</v>
+      </c>
+      <c r="X9" t="n">
+        <v>24.22755349018178</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>11.38529810400037</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>0.3590201065011612</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C10" t="n">
         <v>0.06642947158209415</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>0.2988888888888889</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E10" t="n">
         <v>0.4418538881768926</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F10" t="n">
         <v>166.0177140491317</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G10" t="n">
         <v>56.97044445833979</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H10" t="n">
         <v>95.57025253573281</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I10" t="n">
         <v>228.4330970314423</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J10" t="n">
         <v>34.31588296745238</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K10" t="n">
         <v>18.50299478474454</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L10" t="n">
         <v>5</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M10" t="n">
         <v>187.2150349556951</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N10" t="n">
         <v>261.5786998080872</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O10" t="n">
         <v>133.9920618122841</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P10" t="n">
         <v>2.852875557438051</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q10" t="n">
         <v>6.04123289887048</v>
       </c>
-      <c r="R9" t="n">
+      <c r="R10" t="n">
         <v>1.347224826864263</v>
       </c>
-      <c r="S9" t="n">
+      <c r="S10" t="n">
         <v>66.09774053634418</v>
       </c>
-      <c r="T9" t="n">
+      <c r="T10" t="n">
         <v>0.7713599999999999</v>
       </c>
-      <c r="U9" t="n">
+      <c r="U10" t="n">
         <v>0.3030782869161036</v>
       </c>
-      <c r="V9" t="n">
+      <c r="V10" t="n">
         <v>27.60739652580063</v>
       </c>
-      <c r="W9" t="n">
+      <c r="W10" t="n">
         <v>3.910849322327261</v>
       </c>
-      <c r="X9" t="n">
+      <c r="X10" t="n">
         <v>39.291418652264</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Y10" t="n">
         <v>14.16594758825722</v>
       </c>
     </row>

</xml_diff>